<commit_message>
fix: preserve V12 contest result template grouping and repair figure 11 legend
</commit_message>
<xml_diff>
--- a/results/V12/附件5/result1.xlsx
+++ b/results/V12/附件5/result1.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000_ "/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,11 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="宋体"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -56,7 +61,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -64,11 +69,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -86,13 +139,39 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -455,1459 +534,1460 @@
   <dimension ref="A1:B145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14" customHeight="1"/>
   <cols>
-    <col width="13.6328125" customWidth="1" style="5" min="1" max="2"/>
+    <col width="18" customWidth="1" style="5" min="1" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8.7265625" customWidth="1" style="4" min="3" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>时间段</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>购电量</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>00:00-00:10</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="9" t="n">
         <v>1406.6411</v>
       </c>
     </row>
     <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>00:10-00:20</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="9" t="n">
         <v>1406.329866666666</v>
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>00:20-00:30</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>1407.38385</v>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>00:30-00:40</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>1409.07395</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>00:40-00:50</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>1409.80455</v>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>00:50-01:00</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>576.6400166666666</v>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>01:00-01:10</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>577.8597</v>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>01:10-01:20</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>577.9938666666667</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>01:20-01:30</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>911.1613833333331</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>01:30-01:40</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>580.41545</v>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>01:40-01:50</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="9" t="n">
         <v>582.5140166666665</v>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>01:50-02:00</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>583.0740500000001</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>02:00-02:10</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>584.2049166666666</v>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>02:10-02:20</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <v>585.4397833333333</v>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>02:20-02:30</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="9" t="n">
         <v>586.1447499999999</v>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>02:30-02:40</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="9" t="n">
         <v>586.3207666666666</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>02:40-02:50</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <v>586.4253</v>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>02:50-03:00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="9" t="n">
         <v>586.8496</v>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>03:00-03:10</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="9" t="n">
         <v>587.8210166666667</v>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>03:10-03:20</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="9" t="n">
         <v>589.5475666666665</v>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>03:20-03:30</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="9" t="n">
         <v>590.8134666666666</v>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>03:30-03:40</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="9" t="n">
         <v>590.2131166666666</v>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>03:40-03:50</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="9" t="n">
         <v>591.0662666666666</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>03:50-04:00</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n">
+      <c r="B25" s="9" t="n">
         <v>593.3678333333332</v>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>04:00-04:10</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="9" t="n">
         <v>593.6596833333333</v>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>04:10-04:20</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
+      <c r="B27" s="9" t="n">
         <v>592.7863833333333</v>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>04:20-04:30</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="9" t="n">
         <v>593.3378666666665</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>04:30-04:40</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="9" t="n">
         <v>596.6757666666665</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>04:40-04:50</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>597.78025</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>04:50-05:00</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="9" t="n">
         <v>595.1624999999999</v>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>05:00-05:10</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="9" t="n">
         <v>590.6065</v>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>05:10-05:20</t>
         </is>
       </c>
-      <c r="B33" s="8" t="n">
+      <c r="B33" s="9" t="n">
         <v>589.4851833333332</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>05:20-05:30</t>
         </is>
       </c>
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="9" t="n">
         <v>578.4554499999999</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>05:30-05:40</t>
         </is>
       </c>
-      <c r="B35" s="8" t="n">
+      <c r="B35" s="9" t="n">
         <v>1383.659783333333</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>05:40-05:50</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="9" t="n">
         <v>591.1402</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>05:50-06:00</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n">
+      <c r="B37" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>06:00-06:10</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n">
+      <c r="B38" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>06:10-06:20</t>
         </is>
       </c>
-      <c r="B39" s="8" t="n">
+      <c r="B39" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>06:20-06:30</t>
         </is>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>06:30-06:40</t>
         </is>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>06:40-06:50</t>
         </is>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>06:50-07:00</t>
         </is>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B43" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>07:00-07:10</t>
         </is>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>07:10-07:20</t>
         </is>
       </c>
-      <c r="B45" s="8" t="n">
+      <c r="B45" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>07:20-07:30</t>
         </is>
       </c>
-      <c r="B46" s="8" t="n">
+      <c r="B46" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47" ht="14" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>07:30-07:40</t>
         </is>
       </c>
-      <c r="B47" s="8" t="n">
+      <c r="B47" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>07:40-07:50</t>
         </is>
       </c>
-      <c r="B48" s="8" t="n">
+      <c r="B48" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>07:50-08:00</t>
         </is>
       </c>
-      <c r="B49" s="8" t="n">
+      <c r="B49" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>08:00-08:10</t>
         </is>
       </c>
-      <c r="B50" s="8" t="n">
+      <c r="B50" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>08:10-08:20</t>
         </is>
       </c>
-      <c r="B51" s="8" t="n">
+      <c r="B51" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>08:20-08:30</t>
         </is>
       </c>
-      <c r="B52" s="8" t="n">
+      <c r="B52" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>08:30-08:40</t>
         </is>
       </c>
-      <c r="B53" s="8" t="n">
+      <c r="B53" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>08:40-08:50</t>
         </is>
       </c>
-      <c r="B54" s="8" t="n">
+      <c r="B54" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55" ht="14" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>08:50-09:00</t>
         </is>
       </c>
-      <c r="B55" s="8" t="n">
+      <c r="B55" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>09:00-09:10</t>
         </is>
       </c>
-      <c r="B56" s="8" t="n">
+      <c r="B56" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>09:10-09:20</t>
         </is>
       </c>
-      <c r="B57" s="8" t="n">
+      <c r="B57" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="58" ht="14" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>09:20-09:30</t>
         </is>
       </c>
-      <c r="B58" s="8" t="n">
+      <c r="B58" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>09:30-09:40</t>
         </is>
       </c>
-      <c r="B59" s="8" t="n">
+      <c r="B59" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>09:40-09:50</t>
         </is>
       </c>
-      <c r="B60" s="8" t="n">
+      <c r="B60" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>09:50-10:00</t>
         </is>
       </c>
-      <c r="B61" s="8" t="n">
+      <c r="B61" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>10:00-10:10</t>
         </is>
       </c>
-      <c r="B62" s="8" t="n">
+      <c r="B62" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>10:10-10:20</t>
         </is>
       </c>
-      <c r="B63" s="8" t="n">
+      <c r="B63" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>10:20-10:30</t>
         </is>
       </c>
-      <c r="B64" s="8" t="n">
+      <c r="B64" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>10:30-10:40</t>
         </is>
       </c>
-      <c r="B65" s="8" t="n">
+      <c r="B65" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>10:40-10:50</t>
         </is>
       </c>
-      <c r="B66" s="8" t="n">
+      <c r="B66" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>10:50-11:00</t>
         </is>
       </c>
-      <c r="B67" s="8" t="n">
+      <c r="B67" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>11:00-11:10</t>
         </is>
       </c>
-      <c r="B68" s="8" t="n">
+      <c r="B68" s="9" t="n">
         <v>575.1709166666665</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>11:10-11:20</t>
         </is>
       </c>
-      <c r="B69" s="8" t="n">
+      <c r="B69" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>11:20-11:30</t>
         </is>
       </c>
-      <c r="B70" s="8" t="n">
+      <c r="B70" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>11:30-11:40</t>
         </is>
       </c>
-      <c r="B71" s="8" t="n">
+      <c r="B71" s="9" t="n">
         <v>179.2771713991827</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
-      <c r="A72" s="5" t="inlineStr">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>11:40-11:50</t>
         </is>
       </c>
-      <c r="B72" s="8" t="n">
+      <c r="B72" s="9" t="n">
         <v>520.1245166666665</v>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>11:50-12:00</t>
         </is>
       </c>
-      <c r="B73" s="8" t="n">
+      <c r="B73" s="9" t="n">
         <v>486.4028999999999</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
-      <c r="A74" s="5" t="inlineStr">
+      <c r="A74" s="7" t="inlineStr">
         <is>
           <t>12:00-12:10</t>
         </is>
       </c>
-      <c r="B74" s="8" t="n">
+      <c r="B74" s="9" t="n">
         <v>480.4124499999999</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="A75" s="7" t="inlineStr">
         <is>
           <t>12:10-12:20</t>
         </is>
       </c>
-      <c r="B75" s="8" t="n">
+      <c r="B75" s="9" t="n">
         <v>485.3</v>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
-      <c r="A76" s="5" t="inlineStr">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>12:20-12:30</t>
         </is>
       </c>
-      <c r="B76" s="8" t="n">
+      <c r="B76" s="9" t="n">
         <v>488.6069666666666</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
-      <c r="A77" s="5" t="inlineStr">
+      <c r="A77" s="7" t="inlineStr">
         <is>
           <t>12:30-12:40</t>
         </is>
       </c>
-      <c r="B77" s="8" t="n">
+      <c r="B77" s="9" t="n">
         <v>498.2707333333332</v>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="A78" s="5" t="inlineStr">
+      <c r="A78" s="7" t="inlineStr">
         <is>
           <t>12:40-12:50</t>
         </is>
       </c>
-      <c r="B78" s="8" t="n">
+      <c r="B78" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
-      <c r="A79" s="5" t="inlineStr">
+      <c r="A79" s="7" t="inlineStr">
         <is>
           <t>12:50-13:00</t>
         </is>
       </c>
-      <c r="B79" s="8" t="n">
+      <c r="B79" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="A80" s="5" t="inlineStr">
+      <c r="A80" s="7" t="inlineStr">
         <is>
           <t>13:00-13:10</t>
         </is>
       </c>
-      <c r="B80" s="8" t="n">
+      <c r="B80" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
-      <c r="A81" s="5" t="inlineStr">
+      <c r="A81" s="7" t="inlineStr">
         <is>
           <t>13:10-13:20</t>
         </is>
       </c>
-      <c r="B81" s="8" t="n">
+      <c r="B81" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="82" ht="14" customHeight="1">
-      <c r="A82" s="5" t="inlineStr">
+      <c r="A82" s="7" t="inlineStr">
         <is>
           <t>13:20-13:30</t>
         </is>
       </c>
-      <c r="B82" s="8" t="n">
+      <c r="B82" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="83" ht="14" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
+      <c r="A83" s="7" t="inlineStr">
         <is>
           <t>13:30-13:40</t>
         </is>
       </c>
-      <c r="B83" s="8" t="n">
+      <c r="B83" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="84" ht="14" customHeight="1">
-      <c r="A84" s="5" t="inlineStr">
+      <c r="A84" s="7" t="inlineStr">
         <is>
           <t>13:40-13:50</t>
         </is>
       </c>
-      <c r="B84" s="8" t="n">
+      <c r="B84" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
-      <c r="A85" s="5" t="inlineStr">
+      <c r="A85" s="7" t="inlineStr">
         <is>
           <t>13:50-14:00</t>
         </is>
       </c>
-      <c r="B85" s="8" t="n">
+      <c r="B85" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
-      <c r="A86" s="5" t="inlineStr">
+      <c r="A86" s="7" t="inlineStr">
         <is>
           <t>14:00-14:10</t>
         </is>
       </c>
-      <c r="B86" s="8" t="n">
+      <c r="B86" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
-      <c r="A87" s="5" t="inlineStr">
+      <c r="A87" s="7" t="inlineStr">
         <is>
           <t>14:10-14:20</t>
         </is>
       </c>
-      <c r="B87" s="8" t="n">
+      <c r="B87" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
-      <c r="A88" s="5" t="inlineStr">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t>14:20-14:30</t>
         </is>
       </c>
-      <c r="B88" s="8" t="n">
+      <c r="B88" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="89" ht="14" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
+      <c r="A89" s="7" t="inlineStr">
         <is>
           <t>14:30-14:40</t>
         </is>
       </c>
-      <c r="B89" s="8" t="n">
+      <c r="B89" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="90" ht="14" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>14:40-14:50</t>
         </is>
       </c>
-      <c r="B90" s="8" t="n">
+      <c r="B90" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="91" ht="14" customHeight="1">
-      <c r="A91" s="5" t="inlineStr">
+      <c r="A91" s="7" t="inlineStr">
         <is>
           <t>14:50-15:00</t>
         </is>
       </c>
-      <c r="B91" s="8" t="n">
+      <c r="B91" s="9" t="n">
         <v>112.0898666666667</v>
       </c>
     </row>
     <row r="92" ht="14" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t>15:00-15:10</t>
         </is>
       </c>
-      <c r="B92" s="8" t="n">
+      <c r="B92" s="9" t="n">
         <v>266.7326936213991</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
-      <c r="A93" s="5" t="inlineStr">
+      <c r="A93" s="7" t="inlineStr">
         <is>
           <t>15:10-15:20</t>
         </is>
       </c>
-      <c r="B93" s="8" t="n">
+      <c r="B93" s="9" t="n">
         <v>197.5235166666666</v>
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
-      <c r="A94" s="5" t="inlineStr">
+      <c r="A94" s="7" t="inlineStr">
         <is>
           <t>15:20-15:30</t>
         </is>
       </c>
-      <c r="B94" s="8" t="n">
+      <c r="B94" s="9" t="n">
         <v>244.8140333333332</v>
       </c>
     </row>
     <row r="95" ht="14" customHeight="1">
-      <c r="A95" s="5" t="inlineStr">
+      <c r="A95" s="7" t="inlineStr">
         <is>
           <t>15:30-15:40</t>
         </is>
       </c>
-      <c r="B95" s="8" t="n">
+      <c r="B95" s="9" t="n">
         <v>295.5346166666667</v>
       </c>
     </row>
     <row r="96" ht="14" customHeight="1">
-      <c r="A96" s="5" t="inlineStr">
+      <c r="A96" s="7" t="inlineStr">
         <is>
           <t>15:40-15:50</t>
         </is>
       </c>
-      <c r="B96" s="8" t="n">
+      <c r="B96" s="9" t="n">
         <v>345.7775000000001</v>
       </c>
     </row>
     <row r="97" ht="14" customHeight="1">
-      <c r="A97" s="5" t="inlineStr">
+      <c r="A97" s="7" t="inlineStr">
         <is>
           <t>15:50-16:00</t>
         </is>
       </c>
-      <c r="B97" s="8" t="n">
+      <c r="B97" s="9" t="n">
         <v>394.9314833333333</v>
       </c>
     </row>
     <row r="98" ht="14" customHeight="1">
-      <c r="A98" s="5" t="inlineStr">
+      <c r="A98" s="7" t="inlineStr">
         <is>
           <t>16:00-16:10</t>
         </is>
       </c>
-      <c r="B98" s="8" t="n">
+      <c r="B98" s="9" t="n">
         <v>445.4316500000001</v>
       </c>
     </row>
     <row r="99" ht="14" customHeight="1">
-      <c r="A99" s="5" t="inlineStr">
+      <c r="A99" s="7" t="inlineStr">
         <is>
           <t>16:10-16:20</t>
         </is>
       </c>
-      <c r="B99" s="8" t="n">
+      <c r="B99" s="9" t="n">
         <v>495.6965833333333</v>
       </c>
     </row>
     <row r="100" ht="14" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
+      <c r="A100" s="7" t="inlineStr">
         <is>
           <t>16:20-16:30</t>
         </is>
       </c>
-      <c r="B100" s="8" t="n">
+      <c r="B100" s="9" t="n">
         <v>547.11905</v>
       </c>
     </row>
     <row r="101" ht="14" customHeight="1">
-      <c r="A101" s="5" t="inlineStr">
+      <c r="A101" s="7" t="inlineStr">
         <is>
           <t>16:30-16:40</t>
         </is>
       </c>
-      <c r="B101" s="8" t="n">
+      <c r="B101" s="9" t="n">
         <v>599.9854333333333</v>
       </c>
     </row>
     <row r="102" ht="14" customHeight="1">
-      <c r="A102" s="5" t="inlineStr">
+      <c r="A102" s="7" t="inlineStr">
         <is>
           <t>16:40-16:50</t>
         </is>
       </c>
-      <c r="B102" s="8" t="n">
+      <c r="B102" s="9" t="n">
         <v>635.4297499999999</v>
       </c>
     </row>
     <row r="103" ht="14" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
+      <c r="A103" s="7" t="inlineStr">
         <is>
           <t>16:50-17:00</t>
         </is>
       </c>
-      <c r="B103" s="8" t="n">
+      <c r="B103" s="9" t="n">
         <v>660.8306833333334</v>
       </c>
     </row>
     <row r="104" ht="14" customHeight="1">
-      <c r="A104" s="5" t="inlineStr">
+      <c r="A104" s="7" t="inlineStr">
         <is>
           <t>17:00-17:10</t>
         </is>
       </c>
-      <c r="B104" s="8" t="n">
+      <c r="B104" s="9" t="n">
         <v>702.0369333333333</v>
       </c>
     </row>
     <row r="105" ht="14" customHeight="1">
-      <c r="A105" s="5" t="inlineStr">
+      <c r="A105" s="7" t="inlineStr">
         <is>
           <t>17:10-17:20</t>
         </is>
       </c>
-      <c r="B105" s="8" t="n">
+      <c r="B105" s="9" t="n">
         <v>738.0657833333332</v>
       </c>
     </row>
     <row r="106" ht="14" customHeight="1">
-      <c r="A106" s="5" t="inlineStr">
+      <c r="A106" s="7" t="inlineStr">
         <is>
           <t>17:20-17:30</t>
         </is>
       </c>
-      <c r="B106" s="8" t="n">
+      <c r="B106" s="9" t="n">
         <v>775.9447166666665</v>
       </c>
     </row>
     <row r="107" ht="14" customHeight="1">
-      <c r="A107" s="5" t="inlineStr">
+      <c r="A107" s="7" t="inlineStr">
         <is>
           <t>17:30-17:40</t>
         </is>
       </c>
-      <c r="B107" s="8" t="n">
+      <c r="B107" s="9" t="n">
         <v>826.08325</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1">
-      <c r="A108" s="5" t="inlineStr">
+      <c r="A108" s="7" t="inlineStr">
         <is>
           <t>17:40-17:50</t>
         </is>
       </c>
-      <c r="B108" s="8" t="n">
+      <c r="B108" s="9" t="n">
         <v>762.4227999999998</v>
       </c>
     </row>
     <row r="109" ht="14" customHeight="1">
-      <c r="A109" s="5" t="inlineStr">
+      <c r="A109" s="7" t="inlineStr">
         <is>
           <t>17:50-18:00</t>
         </is>
       </c>
-      <c r="B109" s="8" t="n">
+      <c r="B109" s="9" t="n">
         <v>636.9826166666667</v>
       </c>
     </row>
     <row r="110" ht="14" customHeight="1">
-      <c r="A110" s="5" t="inlineStr">
+      <c r="A110" s="7" t="inlineStr">
         <is>
           <t>18:00-18:10</t>
         </is>
       </c>
-      <c r="B110" s="8" t="n">
+      <c r="B110" s="9" t="n">
         <v>531.8940499999999</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
-      <c r="A111" s="5" t="inlineStr">
+      <c r="A111" s="7" t="inlineStr">
         <is>
           <t>18:10-18:20</t>
         </is>
       </c>
-      <c r="B111" s="8" t="n">
+      <c r="B111" s="9" t="n">
         <v>678.8305333333333</v>
       </c>
     </row>
     <row r="112" ht="14" customHeight="1">
-      <c r="A112" s="5" t="inlineStr">
+      <c r="A112" s="7" t="inlineStr">
         <is>
           <t>18:20-18:30</t>
         </is>
       </c>
-      <c r="B112" s="8" t="n">
+      <c r="B112" s="9" t="n">
         <v>686.2684999999999</v>
       </c>
     </row>
     <row r="113" ht="14" customHeight="1">
-      <c r="A113" s="5" t="inlineStr">
+      <c r="A113" s="7" t="inlineStr">
         <is>
           <t>18:30-18:40</t>
         </is>
       </c>
-      <c r="B113" s="8" t="n">
+      <c r="B113" s="9" t="n">
         <v>696.5043833333333</v>
       </c>
     </row>
     <row r="114" ht="14" customHeight="1">
-      <c r="A114" s="5" t="inlineStr">
+      <c r="A114" s="7" t="inlineStr">
         <is>
           <t>18:40-18:50</t>
         </is>
       </c>
-      <c r="B114" s="8" t="n">
+      <c r="B114" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="115" ht="14" customHeight="1">
-      <c r="A115" s="5" t="inlineStr">
+      <c r="A115" s="7" t="inlineStr">
         <is>
           <t>18:50-19:00</t>
         </is>
       </c>
-      <c r="B115" s="8" t="n">
+      <c r="B115" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="116" ht="14" customHeight="1">
-      <c r="A116" s="5" t="inlineStr">
+      <c r="A116" s="7" t="inlineStr">
         <is>
           <t>19:00-19:10</t>
         </is>
       </c>
-      <c r="B116" s="8" t="n">
+      <c r="B116" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="117" ht="14" customHeight="1">
-      <c r="A117" s="5" t="inlineStr">
+      <c r="A117" s="7" t="inlineStr">
         <is>
           <t>19:10-19:20</t>
         </is>
       </c>
-      <c r="B117" s="8" t="n">
+      <c r="B117" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="118" ht="14" customHeight="1">
-      <c r="A118" s="5" t="inlineStr">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t>19:20-19:30</t>
         </is>
       </c>
-      <c r="B118" s="8" t="n">
+      <c r="B118" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="119" ht="14" customHeight="1">
-      <c r="A119" s="5" t="inlineStr">
+      <c r="A119" s="7" t="inlineStr">
         <is>
           <t>19:30-19:40</t>
         </is>
       </c>
-      <c r="B119" s="8" t="n">
+      <c r="B119" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="120" ht="14" customHeight="1">
-      <c r="A120" s="5" t="inlineStr">
+      <c r="A120" s="7" t="inlineStr">
         <is>
           <t>19:40-19:50</t>
         </is>
       </c>
-      <c r="B120" s="8" t="n">
+      <c r="B120" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="121" ht="14" customHeight="1">
-      <c r="A121" s="5" t="inlineStr">
+      <c r="A121" s="7" t="inlineStr">
         <is>
           <t>19:50-20:00</t>
         </is>
       </c>
-      <c r="B121" s="8" t="n">
+      <c r="B121" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="122" ht="14" customHeight="1">
-      <c r="A122" s="5" t="inlineStr">
+      <c r="A122" s="7" t="inlineStr">
         <is>
           <t>20:00-20:10</t>
         </is>
       </c>
-      <c r="B122" s="8" t="n">
+      <c r="B122" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="123" ht="14" customHeight="1">
-      <c r="A123" s="5" t="inlineStr">
+      <c r="A123" s="7" t="inlineStr">
         <is>
           <t>20:10-20:20</t>
         </is>
       </c>
-      <c r="B123" s="8" t="n">
+      <c r="B123" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="124" ht="14" customHeight="1">
-      <c r="A124" s="5" t="inlineStr">
+      <c r="A124" s="7" t="inlineStr">
         <is>
           <t>20:20-20:30</t>
         </is>
       </c>
-      <c r="B124" s="8" t="n">
+      <c r="B124" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="125" ht="14" customHeight="1">
-      <c r="A125" s="5" t="inlineStr">
+      <c r="A125" s="7" t="inlineStr">
         <is>
           <t>20:30-20:40</t>
         </is>
       </c>
-      <c r="B125" s="8" t="n">
+      <c r="B125" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="126" ht="14" customHeight="1">
-      <c r="A126" s="5" t="inlineStr">
+      <c r="A126" s="7" t="inlineStr">
         <is>
           <t>20:40-20:50</t>
         </is>
       </c>
-      <c r="B126" s="8" t="n">
+      <c r="B126" s="9" t="n">
         <v>715.8689166666666</v>
       </c>
     </row>
     <row r="127" ht="14" customHeight="1">
-      <c r="A127" s="5" t="inlineStr">
+      <c r="A127" s="7" t="inlineStr">
         <is>
           <t>20:50-21:00</t>
         </is>
       </c>
-      <c r="B127" s="8" t="n">
+      <c r="B127" s="9" t="n">
         <v>717.0051166666667</v>
       </c>
     </row>
     <row r="128" ht="14" customHeight="1">
-      <c r="A128" s="5" t="inlineStr">
+      <c r="A128" s="7" t="inlineStr">
         <is>
           <t>21:00-21:10</t>
         </is>
       </c>
-      <c r="B128" s="8" t="n">
+      <c r="B128" s="9" t="n">
         <v>720.1603</v>
       </c>
     </row>
     <row r="129" ht="14" customHeight="1">
-      <c r="A129" s="5" t="inlineStr">
+      <c r="A129" s="7" t="inlineStr">
         <is>
           <t>21:10-21:20</t>
         </is>
       </c>
-      <c r="B129" s="8" t="n">
+      <c r="B129" s="9" t="n">
         <v>717.0548666666666</v>
       </c>
     </row>
     <row r="130" ht="14" customHeight="1">
-      <c r="A130" s="5" t="inlineStr">
+      <c r="A130" s="7" t="inlineStr">
         <is>
           <t>21:20-21:30</t>
         </is>
       </c>
-      <c r="B130" s="8" t="n">
+      <c r="B130" s="9" t="n">
         <v>720.4459666666667</v>
       </c>
     </row>
     <row r="131" ht="14" customHeight="1">
-      <c r="A131" s="5" t="inlineStr">
+      <c r="A131" s="7" t="inlineStr">
         <is>
           <t>21:30-21:40</t>
         </is>
       </c>
-      <c r="B131" s="8" t="n">
+      <c r="B131" s="9" t="n">
         <v>738.1347166666666</v>
       </c>
     </row>
     <row r="132" ht="14" customHeight="1">
-      <c r="A132" s="5" t="inlineStr">
+      <c r="A132" s="7" t="inlineStr">
         <is>
           <t>21:40-21:50</t>
         </is>
       </c>
-      <c r="B132" s="8" t="n">
+      <c r="B132" s="9" t="n">
         <v>671.6935666666666</v>
       </c>
     </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="A133" s="5" t="inlineStr">
+      <c r="A133" s="7" t="inlineStr">
         <is>
           <t>21:50-22:00</t>
         </is>
       </c>
-      <c r="B133" s="8" t="n">
+      <c r="B133" s="9" t="n">
         <v>1393.790316666667</v>
       </c>
     </row>
     <row r="134" ht="14" customHeight="1">
-      <c r="A134" s="5" t="inlineStr">
+      <c r="A134" s="7" t="inlineStr">
         <is>
           <t>22:00-22:10</t>
         </is>
       </c>
-      <c r="B134" s="8" t="n">
+      <c r="B134" s="9" t="n">
         <v>1384.8989</v>
       </c>
     </row>
     <row r="135" ht="14" customHeight="1">
-      <c r="A135" s="5" t="inlineStr">
+      <c r="A135" s="7" t="inlineStr">
         <is>
           <t>22:10-22:20</t>
         </is>
       </c>
-      <c r="B135" s="8" t="n">
+      <c r="B135" s="9" t="n">
         <v>568.8260499999999</v>
       </c>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="A136" s="5" t="inlineStr">
+      <c r="A136" s="7" t="inlineStr">
         <is>
           <t>22:20-22:30</t>
         </is>
       </c>
-      <c r="B136" s="8" t="n">
+      <c r="B136" s="9" t="n">
         <v>1396.98855</v>
       </c>
     </row>
     <row r="137" ht="14" customHeight="1">
-      <c r="A137" s="5" t="inlineStr">
+      <c r="A137" s="7" t="inlineStr">
         <is>
           <t>22:30-22:40</t>
         </is>
       </c>
-      <c r="B137" s="8" t="n">
+      <c r="B137" s="9" t="n">
         <v>1397.759866666666</v>
       </c>
     </row>
     <row r="138" ht="14" customHeight="1">
-      <c r="A138" s="5" t="inlineStr">
+      <c r="A138" s="7" t="inlineStr">
         <is>
           <t>22:40-22:50</t>
         </is>
       </c>
-      <c r="B138" s="8" t="n">
+      <c r="B138" s="9" t="n">
         <v>566.7474333333332</v>
       </c>
     </row>
     <row r="139" ht="14" customHeight="1">
-      <c r="A139" s="5" t="inlineStr">
+      <c r="A139" s="7" t="inlineStr">
         <is>
           <t>22:50-23:00</t>
         </is>
       </c>
-      <c r="B139" s="8" t="n">
+      <c r="B139" s="9" t="n">
         <v>1399.873766666667</v>
       </c>
     </row>
     <row r="140" ht="14" customHeight="1">
-      <c r="A140" s="5" t="inlineStr">
+      <c r="A140" s="7" t="inlineStr">
         <is>
           <t>23:00-23:10</t>
         </is>
       </c>
-      <c r="B140" s="8" t="n">
+      <c r="B140" s="9" t="n">
         <v>567.83015</v>
       </c>
     </row>
     <row r="141" ht="14" customHeight="1">
-      <c r="A141" s="5" t="inlineStr">
+      <c r="A141" s="7" t="inlineStr">
         <is>
           <t>23:10-23:20</t>
         </is>
       </c>
-      <c r="B141" s="8" t="n">
+      <c r="B141" s="9" t="n">
         <v>902.6919666666664</v>
       </c>
     </row>
     <row r="142" ht="14" customHeight="1">
-      <c r="A142" s="5" t="inlineStr">
+      <c r="A142" s="7" t="inlineStr">
         <is>
           <t>23:20-23:30</t>
         </is>
       </c>
-      <c r="B142" s="8" t="n">
+      <c r="B142" s="9" t="n">
         <v>1403.663516666667</v>
       </c>
     </row>
     <row r="143" ht="14" customHeight="1">
-      <c r="A143" s="5" t="inlineStr">
+      <c r="A143" s="7" t="inlineStr">
         <is>
           <t>23:30-23:40</t>
         </is>
       </c>
-      <c r="B143" s="8" t="n">
+      <c r="B143" s="9" t="n">
         <v>571.6153833333333</v>
       </c>
     </row>
     <row r="144" ht="14" customHeight="1">
-      <c r="A144" s="5" t="inlineStr">
+      <c r="A144" s="7" t="inlineStr">
         <is>
           <t>23:40-23:50</t>
         </is>
       </c>
-      <c r="B144" s="8" t="n">
+      <c r="B144" s="9" t="n">
         <v>573.1768333333333</v>
       </c>
     </row>
     <row r="145" ht="14" customHeight="1">
-      <c r="A145" s="5" t="inlineStr">
+      <c r="A145" s="7" t="inlineStr">
         <is>
           <t>23:50-24:00</t>
         </is>
       </c>
-      <c r="B145" s="8" t="n">
+      <c r="B145" s="9" t="n">
         <v>574.1209833333332</v>
       </c>
     </row>
@@ -1926,130 +2006,141 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14" customHeight="1"/>
   <cols>
-    <col width="11.6328125" customWidth="1" style="4" min="1" max="3"/>
-    <col width="8.7265625" customWidth="1" style="4" min="4" max="16384"/>
+    <col width="18" customWidth="1" style="4" min="1" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" style="4" min="4" max="16384"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>时间段</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>充电量</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>放电量</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>时刻</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>储电量</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>0:00-4:00</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="11" t="n">
         <v>4499.999999999999</v>
       </c>
-      <c r="C2" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="11" t="n">
         <v>6000</v>
       </c>
     </row>
     <row r="3" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>4:00-8:00</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="14" t="n">
         <v>833.3333333333331</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="14" t="n">
         <v>6365.8412</v>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>24:00</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="14" t="n">
         <v>6000</v>
       </c>
     </row>
     <row r="4" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>8:00-12:00</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="14" t="n">
         <v>4787.964288065848</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="14" t="n">
         <v>1702.996983333333</v>
       </c>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
     </row>
     <row r="5" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>12:00-16:00</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="14" t="n">
         <v>5286.035176954731</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="14" t="n">
         <v>91.1013833333335</v>
       </c>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
     </row>
     <row r="6" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>16:00-20:00</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="9" t="n">
+      <c r="B6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="14" t="n">
         <v>5780.131883333333</v>
       </c>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="13" t="n"/>
     </row>
     <row r="7" ht="14" customFormat="1" customHeight="1" s="5">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>20:00-24:00</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="17" t="n">
         <v>5333.333333333332</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="17" t="n">
         <v>2859.868116666667</v>
       </c>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>